<commit_message>
Cambios correspondientes a Entrega Final
</commit_message>
<xml_diff>
--- a/Recursos/Importar/plantilla_listadoConvenios.xlsx
+++ b/Recursos/Importar/plantilla_listadoConvenios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\pruebas\Recursos\Importar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF3DF7E9-000F-430C-B2EF-CE557FEF2D1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F312FD6-65AA-4C8B-9073-9A19AFF0BFED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>Nº CONV.</t>
   </si>
@@ -79,19 +79,16 @@
     <t>28001</t>
   </si>
   <si>
-    <t>910000000</t>
-  </si>
-  <si>
     <t>Juan Pérez López</t>
   </si>
   <si>
-    <t>DAW</t>
-  </si>
-  <si>
     <t>01.01.25</t>
   </si>
   <si>
     <t>01.01.27</t>
+  </si>
+  <si>
+    <t>DAW 2º</t>
   </si>
 </sst>
 </file>
@@ -107,20 +104,19 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
-      <sz val="9"/>
-      <color rgb="FF888888"/>
+      <b/>
+      <sz val="8"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF9C5700"/>
-      <name val="Calibri"/>
+      <sz val="8"/>
+      <color indexed="10"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -129,7 +125,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
+        <fgColor indexed="51"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -143,33 +146,51 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFCCCCCC"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color rgb="FFCCCCCC"/>
+        <color indexed="64"/>
       </right>
-      <top/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
       <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Neutral" xfId="1" builtinId="28"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -488,22 +509,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="2" t="s">
@@ -512,13 +533,13 @@
       <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
       <c r="L1" s="2" t="s">
@@ -529,41 +550,41 @@
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="6">
+        <v>910000000</v>
+      </c>
+      <c r="H2" s="6"/>
+      <c r="I2" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K2" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="L2" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="K2" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M2" s="1"/>
+      <c r="M2" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>